<commit_message>
Fix horizontal alignment of template remarks field.
</commit_message>
<xml_diff>
--- a/src/main/resources/com/develhack/ddiff/reporter/template.xlsx
+++ b/src/main/resources/com/develhack/ddiff/reporter/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yosuk\git\ddiff-reporter-excel\src\main\resources\com\develhack\ddiff\reporter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E844E05-C130-4845-9F14-52F259B682DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81561F5B-4E9B-49BC-ADCD-AA399C8187A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="37680" windowHeight="24480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -200,14 +200,7 @@
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEEEEE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill>
@@ -236,36 +229,9 @@
       </font>
     </dxf>
     <dxf>
-      <font>
-        <u/>
-        <color theme="8" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFEEEEEE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEEEE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEEEFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFEE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -600,26 +566,26 @@
     <row r="3" spans="1:3">
       <c r="A3" s="5"/>
       <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
+      <c r="C3" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <conditionalFormatting sqref="A1:C1048576">
-    <cfRule type="expression" dxfId="9" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="2" stopIfTrue="1">
       <formula>$B1="CHANGED"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="3" stopIfTrue="1">
       <formula>$B1="ADDED"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="4" stopIfTrue="1">
       <formula>$B1="DELETED"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="5" stopIfTrue="1">
       <formula>$B1="UNCOMPARABLE"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$B1="CHANGED"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -668,13 +634,13 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <conditionalFormatting sqref="A1:C1048576">
-    <cfRule type="expression" dxfId="12" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
       <formula>$A1="*"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="6" stopIfTrue="1">
       <formula>$A1="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="7" stopIfTrue="1">
       <formula>$A1="-"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>